<commit_message>
Started 2-nd lab AI
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85BC35AC-3C46-432B-8142-F38E631AECE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4E7C19-77E3-45C3-B00B-FDCF29EDCBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="17">
   <si>
     <t xml:space="preserve">                         Номер работы 
 Название</t>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>Сдана</t>
+  </si>
+  <si>
+    <t>Не существует</t>
+  </si>
+  <si>
+    <t>РГЗ</t>
+  </si>
+  <si>
+    <t>Курсовая</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -107,7 +119,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,6 +147,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -204,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -222,62 +240,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4AF80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7171"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7171"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4AF80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -308,40 +280,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF2F2F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF2F2F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -366,8 +304,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{66754ADA-D36A-490E-B303-DF93166D37E8}" name="Таблица2" displayName="Таблица2" ref="A1:A5" totalsRowShown="0">
-  <autoFilter ref="A1:A5" xr:uid="{66754ADA-D36A-490E-B303-DF93166D37E8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{66754ADA-D36A-490E-B303-DF93166D37E8}" name="Таблица2" displayName="Таблица2" ref="A1:A6" totalsRowShown="0">
+  <autoFilter ref="A1:A6" xr:uid="{66754ADA-D36A-490E-B303-DF93166D37E8}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{D9734E71-C0AB-4E22-A4C3-7E9B46C615F8}" name="Статус"/>
   </tableColumns>
@@ -638,16 +576,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -675,8 +614,17 @@
       <c r="I1" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -699,13 +647,19 @@
         <v>9</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -731,10 +685,16 @@
         <v>9</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -760,15 +720,21 @@
         <v>9</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>9</v>
@@ -786,13 +752,19 @@
         <v>9</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -815,13 +787,19 @@
         <v>9</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -847,10 +825,16 @@
         <v>9</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -878,31 +862,38 @@
       <c r="I8" s="12" t="s">
         <v>9</v>
       </c>
+      <c r="J8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:I8">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+  <conditionalFormatting sqref="B2:K8">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"Не начата"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Начата"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Завершена"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Сдана"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Статус" xr:uid="{4D999426-8380-44EF-BC90-A054C929B5FA}">
           <x14:formula1>
-            <xm:f>Лист1!$A$2:$A$5</xm:f>
+            <xm:f>Лист1!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:I8</xm:sqref>
+          <xm:sqref>B2:K8</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -912,35 +903,40 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IDK nothing really works atp
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4E7C19-77E3-45C3-B00B-FDCF29EDCBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A8D9A1-5571-406C-A1A1-914659EBAB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -247,16 +247,12 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor rgb="FFFF7171"/>
         </patternFill>
       </fill>
     </dxf>
@@ -271,12 +267,16 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7171"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -577,16 +577,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.109375" customWidth="1"/>
-    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.140625" customWidth="1"/>
+    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -624,12 +624,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>9</v>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -694,7 +694,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -729,7 +729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -737,7 +737,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>9</v>
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -799,7 +799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -834,12 +834,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>9</v>
@@ -871,17 +871,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:K8">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"Не начата"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"Сдана"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"Завершена"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"Начата"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"Завершена"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Сдана"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+      <formula>"Не начата"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -904,37 +904,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Lab 1 CrossPP completed
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A8D9A1-5571-406C-A1A1-914659EBAB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B90EF7-D526-4240-9956-E103EAEDD8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -577,16 +577,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.140625" customWidth="1"/>
-    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -624,7 +624,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -694,7 +694,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -729,7 +729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -799,12 +799,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>9</v>
@@ -834,7 +834,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -904,37 +904,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Start 2 lab crossPP
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B90EF7-D526-4240-9956-E103EAEDD8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0184D949-A1CC-4577-AF5A-F64A2DD41570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -577,16 +577,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.109375" customWidth="1"/>
-    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.140625" customWidth="1"/>
+    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -624,7 +624,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -694,7 +694,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -729,7 +729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -799,7 +799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -807,7 +807,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>9</v>
@@ -834,7 +834,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -904,37 +904,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Almost done 3 CrossPP
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{556396B8-1195-472D-8737-5DE3ACA47DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113F307E-D2D6-4210-95C6-84F03B316935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -810,7 +810,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
AIS mostly done and some of AI 2 lab done
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DFC9E0-EC40-4C17-940B-1460F61D846C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9857C1D-932F-42A5-B15C-BCD768215498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -577,16 +577,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.140625" customWidth="1"/>
-    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -624,7 +624,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -694,12 +694,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>9</v>
@@ -729,7 +729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -775,13 +775,13 @@
         <v>11</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>9</v>
@@ -799,7 +799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -834,7 +834,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -904,37 +904,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Lab 5 AIS half done and TPR 1 lab is done
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9857C1D-932F-42A5-B15C-BCD768215498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F6B79A-35E9-449F-943C-83A6956C2F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -699,7 +699,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Finished AI lab 2 and started lab 3
</commit_message>
<xml_diff>
--- a/Лабораторные работы.xlsx
+++ b/Лабораторные работы.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7-semestr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7 semestr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F6B79A-35E9-449F-943C-83A6956C2F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB8F0EA-D226-41B5-AC44-A1B242E72577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -577,16 +577,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.109375" customWidth="1"/>
-    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.140625" customWidth="1"/>
+    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -624,7 +624,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -694,7 +694,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -729,7 +729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -737,11 +737,11 @@
         <v>12</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>9</v>
-      </c>
       <c r="E5" s="10" t="s">
         <v>9</v>
       </c>
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -799,7 +799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -834,7 +834,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -904,37 +904,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919343F7-CF26-4A7D-98AC-7A889765EA89}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>13</v>
       </c>

</xml_diff>